<commit_message>
Edit results.xlsx on Windows 2026-06-02_16-42
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L50"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -513,25 +513,25 @@
         <v>20260602-143428</v>
       </c>
       <c r="B4" t="str">
-        <v>antennas_opposite</v>
+        <v>antennas_vertical</v>
       </c>
       <c r="C4" t="str">
         <v>3</v>
       </c>
       <c r="D4" t="str">
-        <v>2026-06-02 14:35:18</v>
+        <v>2026-06-02 14:37:11</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-06-02 14:35:31</v>
+        <v>2026-06-02 14:37:19</v>
       </c>
       <c r="F4" t="str">
-        <v>13.24</v>
+        <v>7.52</v>
       </c>
       <c r="G4" t="str">
         <v>9</v>
       </c>
       <c r="H4" t="str">
-        <v>E280117000000217F51E61E7, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E719D, E280117000000217F51E718F, E280117000000217F51E60C4, E2801170000002158BB40D84, E2801170000002158BB40D89</v>
+        <v>E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E60C4, E2801170000002158BB40D89, E280117000000217F51E719A, E280117000000217F51E7194, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E719D</v>
       </c>
       <c r="I4" t="str">
         <v>Source_0, Source_1</v>
@@ -554,25 +554,25 @@
         <v>4</v>
       </c>
       <c r="D5" t="str">
-        <v>2026-06-02 14:37:11</v>
+        <v>2026-06-02 14:38:30</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-06-02 14:37:19</v>
+        <v>2026-06-02 14:39:05</v>
       </c>
       <c r="F5" t="str">
-        <v>7.52</v>
+        <v>35.27</v>
       </c>
       <c r="G5" t="str">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="H5" t="str">
-        <v>E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E60C4, E2801170000002158BB40D89, E280117000000217F51E719A, E280117000000217F51E7194, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E719D</v>
+        <v>E280117000000217F51E61DF, E280117000000217F51E7197, E280117000000217F51E61E4, E280117000000217F51E61E7, E280117000000217F51E61ED, E2801170000002158BB40D89, E280117000000217F51E60C4, E2801170000002158BB40D84, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E719D, E280117000000217F51E7194</v>
       </c>
       <c r="I5" t="str">
         <v>Source_0, Source_1</v>
       </c>
       <c r="K5" t="str">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="L5" t="str">
         <v>100</v>
@@ -589,19 +589,19 @@
         <v>5</v>
       </c>
       <c r="D6" t="str">
-        <v>2026-06-02 14:38:30</v>
+        <v>2026-06-02 14:39:42</v>
       </c>
       <c r="E6" t="str">
-        <v>2026-06-02 14:39:05</v>
+        <v>2026-06-02 14:39:57</v>
       </c>
       <c r="F6" t="str">
-        <v>35.27</v>
+        <v>14.66</v>
       </c>
       <c r="G6" t="str">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H6" t="str">
-        <v>E280117000000217F51E61DF, E280117000000217F51E7197, E280117000000217F51E61E4, E280117000000217F51E61E7, E280117000000217F51E61ED, E2801170000002158BB40D89, E280117000000217F51E60C4, E2801170000002158BB40D84, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E719D, E280117000000217F51E7194</v>
+        <v>E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E60C4, E2801170000002158BB40D84, E280117000000217F51E61E4, E280117000000217F51E61E7, E280117000000217F51E7197, E280117000000217F51E719D, E280117000000217F51E7194, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E719A</v>
       </c>
       <c r="I6" t="str">
         <v>Source_0, Source_1</v>
@@ -610,7 +610,7 @@
         <v>13</v>
       </c>
       <c r="L6" t="str">
-        <v>100</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="7">
@@ -624,19 +624,19 @@
         <v>6</v>
       </c>
       <c r="D7" t="str">
-        <v>2026-06-02 14:39:42</v>
+        <v>2026-06-02 14:44:22</v>
       </c>
       <c r="E7" t="str">
-        <v>2026-06-02 14:39:57</v>
+        <v>2026-06-02 14:44:34</v>
       </c>
       <c r="F7" t="str">
-        <v>14.66</v>
+        <v>12.64</v>
       </c>
       <c r="G7" t="str">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H7" t="str">
-        <v>E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E60C4, E2801170000002158BB40D84, E280117000000217F51E61E4, E280117000000217F51E61E7, E280117000000217F51E7197, E280117000000217F51E719D, E280117000000217F51E7194, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E719A</v>
+        <v>E2801170000002158BB40D89, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E7194, E280117000000217F51E61E4, E280117000000217F51E7197</v>
       </c>
       <c r="I7" t="str">
         <v>Source_0, Source_1</v>
@@ -645,12 +645,12 @@
         <v>13</v>
       </c>
       <c r="L7" t="str">
-        <v>92.3</v>
+        <v>61.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>20260602-143428</v>
+        <v>20260602-145947</v>
       </c>
       <c r="B8" t="str">
         <v>antennas_vertical</v>
@@ -659,19 +659,19 @@
         <v>7</v>
       </c>
       <c r="D8" t="str">
-        <v>2026-06-02 14:44:22</v>
+        <v>2026-06-02 14:59:57</v>
       </c>
       <c r="E8" t="str">
-        <v>2026-06-02 14:44:34</v>
+        <v>2026-06-02 15:00:13</v>
       </c>
       <c r="F8" t="str">
-        <v>12.64</v>
+        <v>16.76</v>
       </c>
       <c r="G8" t="str">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="H8" t="str">
-        <v>E2801170000002158BB40D89, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E7194, E280117000000217F51E61E4, E280117000000217F51E7197</v>
+        <v>E280117000000217F51E61DF, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E7197, E280117000000217F51E61E7, E280117000000217F51E60C4, E2801170000002158BB40D84, E2801170000002158BB40D89, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E7194, E280117000000217F51E719D, E280117000000217F51E719A</v>
       </c>
       <c r="I8" t="str">
         <v>Source_0, Source_1</v>
@@ -680,7 +680,7 @@
         <v>13</v>
       </c>
       <c r="L8" t="str">
-        <v>61.5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
@@ -694,19 +694,19 @@
         <v>8</v>
       </c>
       <c r="D9" t="str">
-        <v>2026-06-02 14:59:57</v>
+        <v>2026-06-02 15:01:35</v>
       </c>
       <c r="E9" t="str">
-        <v>2026-06-02 15:00:13</v>
+        <v>2026-06-02 15:01:49</v>
       </c>
       <c r="F9" t="str">
-        <v>16.76</v>
+        <v>14.11</v>
       </c>
       <c r="G9" t="str">
         <v>13</v>
       </c>
       <c r="H9" t="str">
-        <v>E280117000000217F51E61DF, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E7197, E280117000000217F51E61E7, E280117000000217F51E60C4, E2801170000002158BB40D84, E2801170000002158BB40D89, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E7194, E280117000000217F51E719D, E280117000000217F51E719A</v>
+        <v>E2801170000002158BB40D89, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E719D, E280117000000217F51E7194, E280117000000217F51E61DF, E2801170000002158BB40D84, E280117000000217F51E61ED, E280117000000217F51E61E4, E280117000000217F51E61E7, E280117000000217F51E7197, E280117000000217F51E60C4</v>
       </c>
       <c r="I9" t="str">
         <v>Source_0, Source_1</v>
@@ -729,19 +729,19 @@
         <v>9</v>
       </c>
       <c r="D10" t="str">
-        <v>2026-06-02 15:01:35</v>
+        <v>2026-06-02 15:03:11</v>
       </c>
       <c r="E10" t="str">
-        <v>2026-06-02 15:01:49</v>
+        <v>2026-06-02 15:03:26</v>
       </c>
       <c r="F10" t="str">
-        <v>14.11</v>
+        <v>14.47</v>
       </c>
       <c r="G10" t="str">
         <v>13</v>
       </c>
       <c r="H10" t="str">
-        <v>E2801170000002158BB40D89, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E719D, E280117000000217F51E7194, E280117000000217F51E61DF, E2801170000002158BB40D84, E280117000000217F51E61ED, E280117000000217F51E61E4, E280117000000217F51E61E7, E280117000000217F51E7197, E280117000000217F51E60C4</v>
+        <v>E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E60C4, E280117000000217F51E61DF, E280117000000217F51E7197, E2801170000002158BB40D89, E280117000000217F51E61E7, E280117000000217F51E7194, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E719D, E2801170000002158BB40D84</v>
       </c>
       <c r="I10" t="str">
         <v>Source_0, Source_1</v>
@@ -764,19 +764,19 @@
         <v>10</v>
       </c>
       <c r="D11" t="str">
-        <v>2026-06-02 15:03:11</v>
+        <v>2026-06-02 15:03:52</v>
       </c>
       <c r="E11" t="str">
-        <v>2026-06-02 15:03:26</v>
+        <v>2026-06-02 15:04:03</v>
       </c>
       <c r="F11" t="str">
-        <v>14.47</v>
+        <v>10.48</v>
       </c>
       <c r="G11" t="str">
         <v>13</v>
       </c>
       <c r="H11" t="str">
-        <v>E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E60C4, E280117000000217F51E61DF, E280117000000217F51E7197, E2801170000002158BB40D89, E280117000000217F51E61E7, E280117000000217F51E7194, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E719D, E2801170000002158BB40D84</v>
+        <v>E2801170000002158BB40D89, E280117000000217F51E7197, E280117000000217F51E61DF, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E719D, E280117000000217F51E7194, E280117000000217F51E61E7, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E60C4, E2801170000002158BB40D84</v>
       </c>
       <c r="I11" t="str">
         <v>Source_0, Source_1</v>
@@ -799,19 +799,19 @@
         <v>11</v>
       </c>
       <c r="D12" t="str">
-        <v>2026-06-02 15:03:52</v>
+        <v>2026-06-02 15:04:55</v>
       </c>
       <c r="E12" t="str">
-        <v>2026-06-02 15:04:03</v>
+        <v>2026-06-02 15:05:09</v>
       </c>
       <c r="F12" t="str">
-        <v>10.48</v>
+        <v>14.37</v>
       </c>
       <c r="G12" t="str">
         <v>13</v>
       </c>
       <c r="H12" t="str">
-        <v>E2801170000002158BB40D89, E280117000000217F51E7197, E280117000000217F51E61DF, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E719D, E280117000000217F51E7194, E280117000000217F51E61E7, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E60C4, E2801170000002158BB40D84</v>
+        <v>E280117000000217F51E61ED, E280117000000217F51E61DF, E280117000000217F51E60C4, E280117000000217F51E61E7, E2801170000002158BB40D84, E280117000000217F51E61E4, E2801170000002158BB40D89, E280117000000217F51E7197, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E7194</v>
       </c>
       <c r="I12" t="str">
         <v>Source_0, Source_1</v>
@@ -834,19 +834,19 @@
         <v>12</v>
       </c>
       <c r="D13" t="str">
-        <v>2026-06-02 15:04:55</v>
+        <v>2026-06-02 15:05:39</v>
       </c>
       <c r="E13" t="str">
-        <v>2026-06-02 15:05:09</v>
+        <v>2026-06-02 15:05:52</v>
       </c>
       <c r="F13" t="str">
-        <v>14.37</v>
+        <v>12.91</v>
       </c>
       <c r="G13" t="str">
         <v>13</v>
       </c>
       <c r="H13" t="str">
-        <v>E280117000000217F51E61ED, E280117000000217F51E61DF, E280117000000217F51E60C4, E280117000000217F51E61E7, E2801170000002158BB40D84, E280117000000217F51E61E4, E2801170000002158BB40D89, E280117000000217F51E7197, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E7194</v>
+        <v>E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E718F, E280117000000217F51E7197, E280117000000217F51E61ED, E2801170000002158BB40D89, E2801170000002158BB40D84, E280117000000217F51E61E4, E280117000000217F51E60C4, E280117000000217F51E61E7, E280117000000217F51E61DF</v>
       </c>
       <c r="I13" t="str">
         <v>Source_0, Source_1</v>
@@ -869,19 +869,19 @@
         <v>13</v>
       </c>
       <c r="D14" t="str">
-        <v>2026-06-02 15:05:39</v>
+        <v>2026-06-02 15:06:19</v>
       </c>
       <c r="E14" t="str">
-        <v>2026-06-02 15:05:52</v>
+        <v>2026-06-02 15:06:58</v>
       </c>
       <c r="F14" t="str">
-        <v>12.91</v>
+        <v>39.34</v>
       </c>
       <c r="G14" t="str">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="H14" t="str">
-        <v>E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E718F, E280117000000217F51E7197, E280117000000217F51E61ED, E2801170000002158BB40D89, E2801170000002158BB40D84, E280117000000217F51E61E4, E280117000000217F51E60C4, E280117000000217F51E61E7, E280117000000217F51E61DF</v>
+        <v>E280117000000217F51E61DF, E280117000000217F51E7197, E280117000000217F51E61E4, E280117000000217F51E719D, E280117000000217F51E61ED, E280117000000217F51E60C4, E280117000000217F51E7194</v>
       </c>
       <c r="I14" t="str">
         <v>Source_0, Source_1</v>
@@ -890,7 +890,7 @@
         <v>13</v>
       </c>
       <c r="L14" t="str">
-        <v>100</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="15">
@@ -904,19 +904,19 @@
         <v>14</v>
       </c>
       <c r="D15" t="str">
-        <v>2026-06-02 15:06:19</v>
+        <v>2026-06-02 15:07:36</v>
       </c>
       <c r="E15" t="str">
-        <v>2026-06-02 15:06:58</v>
+        <v>2026-06-02 15:07:48</v>
       </c>
       <c r="F15" t="str">
-        <v>39.34</v>
+        <v>12.29</v>
       </c>
       <c r="G15" t="str">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="H15" t="str">
-        <v>E280117000000217F51E61DF, E280117000000217F51E7197, E280117000000217F51E61E4, E280117000000217F51E719D, E280117000000217F51E61ED, E280117000000217F51E60C4, E280117000000217F51E7194</v>
+        <v>E280117000000217F51E61E7, E280117000000217F51E61E4, E280117000000217F51E7197, E280117000000217F51E61ED, E280117000000217F51E60C4, E2801170000002158BB40D89, E2801170000002158BB40D84, E280117000000217F51E61DF, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E7082, E280117000000217F51E7194</v>
       </c>
       <c r="I15" t="str">
         <v>Source_0, Source_1</v>
@@ -925,7 +925,7 @@
         <v>13</v>
       </c>
       <c r="L15" t="str">
-        <v>53.8</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16">
@@ -939,19 +939,19 @@
         <v>15</v>
       </c>
       <c r="D16" t="str">
-        <v>2026-06-02 15:07:36</v>
+        <v>2026-06-02 15:08:18</v>
       </c>
       <c r="E16" t="str">
-        <v>2026-06-02 15:07:48</v>
+        <v>2026-06-02 15:08:34</v>
       </c>
       <c r="F16" t="str">
-        <v>12.29</v>
+        <v>15.54</v>
       </c>
       <c r="G16" t="str">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H16" t="str">
-        <v>E280117000000217F51E61E7, E280117000000217F51E61E4, E280117000000217F51E7197, E280117000000217F51E61ED, E280117000000217F51E60C4, E2801170000002158BB40D89, E2801170000002158BB40D84, E280117000000217F51E61DF, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E7082, E280117000000217F51E7194</v>
+        <v>E280117000000217F51E60C4, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E61E7, E2801170000002158BB40D84, E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E61E4, E280117000000217F51E61ED</v>
       </c>
       <c r="I16" t="str">
         <v>Source_0, Source_1</v>
@@ -960,7 +960,7 @@
         <v>13</v>
       </c>
       <c r="L16" t="str">
-        <v>100</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="17">
@@ -974,19 +974,19 @@
         <v>16</v>
       </c>
       <c r="D17" t="str">
-        <v>2026-06-02 15:08:18</v>
+        <v>2026-06-02 15:09:01</v>
       </c>
       <c r="E17" t="str">
-        <v>2026-06-02 15:08:34</v>
+        <v>2026-06-02 15:09:15</v>
       </c>
       <c r="F17" t="str">
-        <v>15.54</v>
+        <v>13.68</v>
       </c>
       <c r="G17" t="str">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H17" t="str">
-        <v>E280117000000217F51E60C4, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E61E7, E2801170000002158BB40D84, E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E61E4, E280117000000217F51E61ED</v>
+        <v>E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E7197, E280117000000217F51E61E4, E280117000000217F51E61E7, E280117000000217F51E61ED, E2801170000002158BB40D84, E280117000000217F51E60C4, E280117000000217F51E719D, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E718F</v>
       </c>
       <c r="I17" t="str">
         <v>Source_0, Source_1</v>
@@ -995,7 +995,7 @@
         <v>13</v>
       </c>
       <c r="L17" t="str">
-        <v>92.3</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18">
@@ -1009,19 +1009,19 @@
         <v>17</v>
       </c>
       <c r="D18" t="str">
-        <v>2026-06-02 15:09:01</v>
+        <v>2026-06-02 15:09:49</v>
       </c>
       <c r="E18" t="str">
-        <v>2026-06-02 15:09:15</v>
+        <v>2026-06-02 15:10:02</v>
       </c>
       <c r="F18" t="str">
-        <v>13.68</v>
+        <v>12.84</v>
       </c>
       <c r="G18" t="str">
         <v>13</v>
       </c>
       <c r="H18" t="str">
-        <v>E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E7197, E280117000000217F51E61E4, E280117000000217F51E61E7, E280117000000217F51E61ED, E2801170000002158BB40D84, E280117000000217F51E60C4, E280117000000217F51E719D, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E718F</v>
+        <v>E280117000000217F51E61DF, E280117000000217F51E60C4, E2801170000002158BB40D89, E280117000000217F51E61E7, E280117000000217F51E61ED, E280117000000217F51E61E4, E280117000000217F51E7197, E2801170000002158BB40D84, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E718F</v>
       </c>
       <c r="I18" t="str">
         <v>Source_0, Source_1</v>
@@ -1044,19 +1044,19 @@
         <v>18</v>
       </c>
       <c r="D19" t="str">
-        <v>2026-06-02 15:09:49</v>
+        <v>2026-06-02 15:10:27</v>
       </c>
       <c r="E19" t="str">
-        <v>2026-06-02 15:10:02</v>
+        <v>2026-06-02 15:10:43</v>
       </c>
       <c r="F19" t="str">
-        <v>12.84</v>
+        <v>15.43</v>
       </c>
       <c r="G19" t="str">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H19" t="str">
-        <v>E280117000000217F51E61DF, E280117000000217F51E60C4, E2801170000002158BB40D89, E280117000000217F51E61E7, E280117000000217F51E61ED, E280117000000217F51E61E4, E280117000000217F51E7197, E2801170000002158BB40D84, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E718F</v>
+        <v>E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E61DF, E280117000000217F51E60C4, E2801170000002158BB40D84, E280117000000217F51E61E7, E2801170000002158BB40D89</v>
       </c>
       <c r="I19" t="str">
         <v>Source_0, Source_1</v>
@@ -1065,12 +1065,12 @@
         <v>13</v>
       </c>
       <c r="L19" t="str">
-        <v>100</v>
+        <v>84.6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>20260602-145947</v>
+        <v>20260602-151630</v>
       </c>
       <c r="B20" t="str">
         <v>antennas_vertical</v>
@@ -1079,19 +1079,19 @@
         <v>19</v>
       </c>
       <c r="D20" t="str">
-        <v>2026-06-02 15:10:27</v>
+        <v>2026-06-02 15:17:18</v>
       </c>
       <c r="E20" t="str">
-        <v>2026-06-02 15:10:43</v>
+        <v>2026-06-02 15:17:32</v>
       </c>
       <c r="F20" t="str">
-        <v>15.43</v>
+        <v>14.34</v>
       </c>
       <c r="G20" t="str">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H20" t="str">
-        <v>E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E61DF, E280117000000217F51E60C4, E2801170000002158BB40D84, E280117000000217F51E61E7, E2801170000002158BB40D89</v>
+        <v>E280117000000217F51E61ED, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E7197, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E718F, E280117000000217F51E7194, E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E60C4, E280117000000217F51E61E4</v>
       </c>
       <c r="I20" t="str">
         <v>Source_0, Source_1</v>
@@ -1100,7 +1100,7 @@
         <v>13</v>
       </c>
       <c r="L20" t="str">
-        <v>84.6</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="21">
@@ -1114,19 +1114,19 @@
         <v>20</v>
       </c>
       <c r="D21" t="str">
-        <v>2026-06-02 15:17:18</v>
+        <v>2026-06-02 15:17:59</v>
       </c>
       <c r="E21" t="str">
-        <v>2026-06-02 15:17:32</v>
+        <v>2026-06-02 15:18:19</v>
       </c>
       <c r="F21" t="str">
-        <v>14.34</v>
+        <v>19.28</v>
       </c>
       <c r="G21" t="str">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H21" t="str">
-        <v>E280117000000217F51E61ED, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E7197, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E718F, E280117000000217F51E7194, E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E60C4, E280117000000217F51E61E4</v>
+        <v>E280117000000217F51E61E7, E280117000000217F51E60C4, E280117000000217F51E7197, E2801170000002158BB40D89, E280117000000217F51E61DF, E2801170000002158BB40D84, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E719D, E280117000000217F51E7194</v>
       </c>
       <c r="I21" t="str">
         <v>Source_0, Source_1</v>
@@ -1135,7 +1135,7 @@
         <v>13</v>
       </c>
       <c r="L21" t="str">
-        <v>92.3</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22">
@@ -1149,19 +1149,19 @@
         <v>21</v>
       </c>
       <c r="D22" t="str">
-        <v>2026-06-02 15:17:59</v>
+        <v>2026-06-02 15:19:11</v>
       </c>
       <c r="E22" t="str">
-        <v>2026-06-02 15:18:19</v>
+        <v>2026-06-02 15:19:25</v>
       </c>
       <c r="F22" t="str">
-        <v>19.28</v>
+        <v>14.05</v>
       </c>
       <c r="G22" t="str">
         <v>13</v>
       </c>
       <c r="H22" t="str">
-        <v>E280117000000217F51E61E7, E280117000000217F51E60C4, E280117000000217F51E7197, E2801170000002158BB40D89, E280117000000217F51E61DF, E2801170000002158BB40D84, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E719D, E280117000000217F51E7194</v>
+        <v>E280117000000217F51E61ED, E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E7197, E280117000000217F51E61E4, E280117000000217F51E60C4, E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E718F</v>
       </c>
       <c r="I22" t="str">
         <v>Source_0, Source_1</v>
@@ -1175,7 +1175,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>20260602-151630</v>
+        <v>20260602-152458</v>
       </c>
       <c r="B23" t="str">
         <v>antennas_vertical</v>
@@ -1184,19 +1184,19 @@
         <v>22</v>
       </c>
       <c r="D23" t="str">
-        <v>2026-06-02 15:19:11</v>
+        <v>2026-06-02 15:25:14</v>
       </c>
       <c r="E23" t="str">
-        <v>2026-06-02 15:19:25</v>
+        <v>2026-06-02 15:25:32</v>
       </c>
       <c r="F23" t="str">
-        <v>14.05</v>
+        <v>17.96</v>
       </c>
       <c r="G23" t="str">
         <v>13</v>
       </c>
       <c r="H23" t="str">
-        <v>E280117000000217F51E61ED, E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E7197, E280117000000217F51E61E4, E280117000000217F51E60C4, E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E718F</v>
+        <v>E280117000000217F51E61E7, E280117000000217F51E7197, E280117000000217F51E61E4, E280117000000217F51E60C4, E2801170000002158BB40D84, E280117000000217F51E61ED, E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E718F, E280117000000217F51E719D</v>
       </c>
       <c r="I23" t="str">
         <v>Source_0, Source_1</v>
@@ -1219,19 +1219,19 @@
         <v>23</v>
       </c>
       <c r="D24" t="str">
-        <v>2026-06-02 15:25:14</v>
+        <v>2026-06-02 15:26:20</v>
       </c>
       <c r="E24" t="str">
-        <v>2026-06-02 15:25:32</v>
+        <v>2026-06-02 15:26:32</v>
       </c>
       <c r="F24" t="str">
-        <v>17.96</v>
+        <v>11.93</v>
       </c>
       <c r="G24" t="str">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H24" t="str">
-        <v>E280117000000217F51E61E7, E280117000000217F51E7197, E280117000000217F51E61E4, E280117000000217F51E60C4, E2801170000002158BB40D84, E280117000000217F51E61ED, E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E718F, E280117000000217F51E719D</v>
+        <v>E2801170000002158BB40D89, E280117000000217F51E61ED, E280117000000217F51E61E4, E280117000000217F51E60C4, E280117000000217F51E61E7, E2801170000002158BB40D84, E280117000000217F51E719A, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E61DF</v>
       </c>
       <c r="I24" t="str">
         <v>Source_0, Source_1</v>
@@ -1240,7 +1240,7 @@
         <v>13</v>
       </c>
       <c r="L24" t="str">
-        <v>100</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="25">
@@ -1254,19 +1254,19 @@
         <v>24</v>
       </c>
       <c r="D25" t="str">
-        <v>2026-06-02 15:26:20</v>
+        <v>2026-06-02 15:28:02</v>
       </c>
       <c r="E25" t="str">
-        <v>2026-06-02 15:26:32</v>
+        <v>2026-06-02 15:28:17</v>
       </c>
       <c r="F25" t="str">
-        <v>11.93</v>
+        <v>15.5</v>
       </c>
       <c r="G25" t="str">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H25" t="str">
-        <v>E2801170000002158BB40D89, E280117000000217F51E61ED, E280117000000217F51E61E4, E280117000000217F51E60C4, E280117000000217F51E61E7, E2801170000002158BB40D84, E280117000000217F51E719A, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E61DF</v>
+        <v>E280117000000217F51E61E4, E280117000000217F51E7197, E280117000000217F51E60C4, E2801170000002158BB40D84, E2801170000002158BB40D89, E280117000000217F51E61E7, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E719D</v>
       </c>
       <c r="I25" t="str">
         <v>Source_0, Source_1</v>
@@ -1275,7 +1275,7 @@
         <v>13</v>
       </c>
       <c r="L25" t="str">
-        <v>92.3</v>
+        <v>84.6</v>
       </c>
     </row>
     <row r="26">
@@ -1289,19 +1289,19 @@
         <v>25</v>
       </c>
       <c r="D26" t="str">
-        <v>2026-06-02 15:28:02</v>
+        <v>2026-06-02 15:28:53</v>
       </c>
       <c r="E26" t="str">
-        <v>2026-06-02 15:28:17</v>
+        <v>2026-06-02 15:29:07</v>
       </c>
       <c r="F26" t="str">
-        <v>15.5</v>
+        <v>13.69</v>
       </c>
       <c r="G26" t="str">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H26" t="str">
-        <v>E280117000000217F51E61E4, E280117000000217F51E7197, E280117000000217F51E60C4, E2801170000002158BB40D84, E2801170000002158BB40D89, E280117000000217F51E61E7, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E719D</v>
+        <v>E2801170000002158BB40D89, E280117000000217F51E61E7, E2801170000002158BB40D84, E280117000000217F51E60C4, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E61DF, E280117000000217F51E61ED, E280117000000217F51E61E4</v>
       </c>
       <c r="I26" t="str">
         <v>Source_0, Source_1</v>
@@ -1310,7 +1310,7 @@
         <v>13</v>
       </c>
       <c r="L26" t="str">
-        <v>84.6</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="27">
@@ -1324,19 +1324,19 @@
         <v>26</v>
       </c>
       <c r="D27" t="str">
-        <v>2026-06-02 15:28:53</v>
+        <v>2026-06-02 15:30:04</v>
       </c>
       <c r="E27" t="str">
-        <v>2026-06-02 15:29:07</v>
+        <v>2026-06-02 15:30:15</v>
       </c>
       <c r="F27" t="str">
-        <v>13.69</v>
+        <v>10.32</v>
       </c>
       <c r="G27" t="str">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H27" t="str">
-        <v>E2801170000002158BB40D89, E280117000000217F51E61E7, E2801170000002158BB40D84, E280117000000217F51E60C4, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E61DF, E280117000000217F51E61ED, E280117000000217F51E61E4</v>
+        <v>E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E61DF, E280117000000217F51E7197, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E7194, E2801170000002158BB40D84, E280117000000217F51E60C4, E280117000000217F51E61E7, E2801170000002158BB40D89</v>
       </c>
       <c r="I27" t="str">
         <v>Source_0, Source_1</v>
@@ -1345,7 +1345,7 @@
         <v>13</v>
       </c>
       <c r="L27" t="str">
-        <v>92.3</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28">
@@ -1359,19 +1359,19 @@
         <v>27</v>
       </c>
       <c r="D28" t="str">
-        <v>2026-06-02 15:30:04</v>
+        <v>2026-06-02 15:30:34</v>
       </c>
       <c r="E28" t="str">
-        <v>2026-06-02 15:30:15</v>
+        <v>2026-06-02 15:30:48</v>
       </c>
       <c r="F28" t="str">
-        <v>10.32</v>
+        <v>13.62</v>
       </c>
       <c r="G28" t="str">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H28" t="str">
-        <v>E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E61DF, E280117000000217F51E7197, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E7194, E2801170000002158BB40D84, E280117000000217F51E60C4, E280117000000217F51E61E7, E2801170000002158BB40D89</v>
+        <v>E2801170000002158BB40D89, E280117000000217F51E61E7, E280117000000217F51E61DF, E2801170000002158BB40D84, E280117000000217F51E60C4, E280117000000217F51E7197, E280117000000217F51E719D, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E61E4</v>
       </c>
       <c r="I28" t="str">
         <v>Source_0, Source_1</v>
@@ -1380,7 +1380,7 @@
         <v>13</v>
       </c>
       <c r="L28" t="str">
-        <v>100</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="29">
@@ -1394,19 +1394,19 @@
         <v>28</v>
       </c>
       <c r="D29" t="str">
-        <v>2026-06-02 15:30:34</v>
+        <v>2026-06-02 15:32:13</v>
       </c>
       <c r="E29" t="str">
-        <v>2026-06-02 15:30:48</v>
+        <v>2026-06-02 15:32:31</v>
       </c>
       <c r="F29" t="str">
-        <v>13.62</v>
+        <v>17.89</v>
       </c>
       <c r="G29" t="str">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H29" t="str">
-        <v>E2801170000002158BB40D89, E280117000000217F51E61E7, E280117000000217F51E61DF, E2801170000002158BB40D84, E280117000000217F51E60C4, E280117000000217F51E7197, E280117000000217F51E719D, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E61E4</v>
+        <v>E280117000000217F51E60C4, E280117000000217F51E61E7, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E7197, E280117000000217F51E61ED, E2801170000002158BB40D84, E280117000000217F51E61DF, E280117000000217F51E61E4, E2801170000002158BB40D89</v>
       </c>
       <c r="I29" t="str">
         <v>Source_0, Source_1</v>
@@ -1415,7 +1415,7 @@
         <v>13</v>
       </c>
       <c r="L29" t="str">
-        <v>92.3</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30">
@@ -1429,19 +1429,19 @@
         <v>29</v>
       </c>
       <c r="D30" t="str">
-        <v>2026-06-02 15:32:13</v>
+        <v>2026-06-02 15:32:57</v>
       </c>
       <c r="E30" t="str">
-        <v>2026-06-02 15:32:31</v>
+        <v>2026-06-02 15:33:09</v>
       </c>
       <c r="F30" t="str">
-        <v>17.89</v>
+        <v>12.82</v>
       </c>
       <c r="G30" t="str">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H30" t="str">
-        <v>E280117000000217F51E60C4, E280117000000217F51E61E7, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E7197, E280117000000217F51E61ED, E2801170000002158BB40D84, E280117000000217F51E61DF, E280117000000217F51E61E4, E2801170000002158BB40D89</v>
+        <v>E280117000000217F51E61DF, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E60C4, E280117000000217F51E7197, E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E7082, E280117000000217F51E719D, E280117000000217F51E7194, E2801170000002158BB40D89</v>
       </c>
       <c r="I30" t="str">
         <v>Source_0, Source_1</v>
@@ -1450,7 +1450,7 @@
         <v>13</v>
       </c>
       <c r="L30" t="str">
-        <v>100</v>
+        <v>84.6</v>
       </c>
     </row>
     <row r="31">
@@ -1464,28 +1464,28 @@
         <v>30</v>
       </c>
       <c r="D31" t="str">
-        <v>2026-06-02 15:32:57</v>
+        <v>2026-06-02 15:34:08</v>
       </c>
       <c r="E31" t="str">
-        <v>2026-06-02 15:33:09</v>
+        <v>2026-06-02 15:34:24</v>
       </c>
       <c r="F31" t="str">
-        <v>12.82</v>
+        <v>15.22</v>
       </c>
       <c r="G31" t="str">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H31" t="str">
-        <v>E280117000000217F51E61DF, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E60C4, E280117000000217F51E7197, E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E7082, E280117000000217F51E719D, E280117000000217F51E7194, E2801170000002158BB40D89</v>
+        <v>E280117000000217F51E61DF, E280117000000217F51E61E7, E2801170000002158BB40D89, E280117000000217F51E61E4, E280117000000217F51E7197, E280117000000217F51E60C4, E2801170000002158BB40D84, E280117000000217F51E61ED, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E7194, E280117000000217F51E7082</v>
       </c>
       <c r="I31" t="str">
         <v>Source_0, Source_1</v>
       </c>
       <c r="K31" t="str">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L31" t="str">
-        <v>84.6</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="32">
@@ -1499,28 +1499,28 @@
         <v>31</v>
       </c>
       <c r="D32" t="str">
-        <v>2026-06-02 15:34:08</v>
+        <v>2026-06-02 15:35:20</v>
       </c>
       <c r="E32" t="str">
-        <v>2026-06-02 15:34:24</v>
+        <v>2026-06-02 15:35:32</v>
       </c>
       <c r="F32" t="str">
-        <v>15.22</v>
+        <v>11.38</v>
       </c>
       <c r="G32" t="str">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H32" t="str">
-        <v>E280117000000217F51E61DF, E280117000000217F51E61E7, E2801170000002158BB40D89, E280117000000217F51E61E4, E280117000000217F51E7197, E280117000000217F51E60C4, E2801170000002158BB40D84, E280117000000217F51E61ED, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E7194, E280117000000217F51E7082</v>
+        <v>E280117000000217F51E7197, E280117000000217F51E60C4, E280117000000217F51E719D, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7194, E280117000000217F51E7082, E280117000000217F51E61DF, E280117000000217F51E61E4, E2801170000002158BB40D89, E280117000000217F51E61E7, E2801170000002158BB40D84</v>
       </c>
       <c r="I32" t="str">
         <v>Source_0, Source_1</v>
       </c>
       <c r="K32" t="str">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L32" t="str">
-        <v>108.3</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="33">
@@ -1534,19 +1534,19 @@
         <v>32</v>
       </c>
       <c r="D33" t="str">
-        <v>2026-06-02 15:35:20</v>
+        <v>2026-06-02 15:36:09</v>
       </c>
       <c r="E33" t="str">
-        <v>2026-06-02 15:35:32</v>
+        <v>2026-06-02 15:36:25</v>
       </c>
       <c r="F33" t="str">
-        <v>11.38</v>
+        <v>15.28</v>
       </c>
       <c r="G33" t="str">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H33" t="str">
-        <v>E280117000000217F51E7197, E280117000000217F51E60C4, E280117000000217F51E719D, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7194, E280117000000217F51E7082, E280117000000217F51E61DF, E280117000000217F51E61E4, E2801170000002158BB40D89, E280117000000217F51E61E7, E2801170000002158BB40D84</v>
+        <v>E2801170000002158BB40D84, E280117000000217F51E60C4, E280117000000217F51E61DF, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E61E7, E2801170000002158BB40D89, E280117000000217F51E7197, E280117000000217F51E7082, E280117000000217F51E719A, E280117000000217F51E7194, E280117000000217F51E718F, E280117000000217F51E719D</v>
       </c>
       <c r="I33" t="str">
         <v>Source_0, Source_1</v>
@@ -1555,7 +1555,7 @@
         <v>13</v>
       </c>
       <c r="L33" t="str">
-        <v>92.3</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34">
@@ -1569,19 +1569,19 @@
         <v>33</v>
       </c>
       <c r="D34" t="str">
-        <v>2026-06-02 15:36:09</v>
+        <v>2026-06-02 15:37:10</v>
       </c>
       <c r="E34" t="str">
-        <v>2026-06-02 15:36:25</v>
+        <v>2026-06-02 15:37:28</v>
       </c>
       <c r="F34" t="str">
-        <v>15.28</v>
+        <v>17.48</v>
       </c>
       <c r="G34" t="str">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H34" t="str">
-        <v>E2801170000002158BB40D84, E280117000000217F51E60C4, E280117000000217F51E61DF, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E61E7, E2801170000002158BB40D89, E280117000000217F51E7197, E280117000000217F51E7082, E280117000000217F51E719A, E280117000000217F51E7194, E280117000000217F51E718F, E280117000000217F51E719D</v>
+        <v>E280117000000217F51E61E7, E280117000000217F51E60C4, E2801170000002158BB40D89, E280117000000217F51E61E4, E280117000000217F51E61DF, E2801170000002158BB40D84, E280117000000217F51E719D, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7194</v>
       </c>
       <c r="I34" t="str">
         <v>Source_0, Source_1</v>
@@ -1590,7 +1590,7 @@
         <v>13</v>
       </c>
       <c r="L34" t="str">
-        <v>100</v>
+        <v>76.9</v>
       </c>
     </row>
     <row r="35">
@@ -1604,19 +1604,19 @@
         <v>34</v>
       </c>
       <c r="D35" t="str">
-        <v>2026-06-02 15:37:10</v>
+        <v>2026-06-02 15:37:57</v>
       </c>
       <c r="E35" t="str">
-        <v>2026-06-02 15:37:28</v>
+        <v>2026-06-02 15:38:12</v>
       </c>
       <c r="F35" t="str">
-        <v>17.48</v>
+        <v>14.34</v>
       </c>
       <c r="G35" t="str">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H35" t="str">
-        <v>E280117000000217F51E61E7, E280117000000217F51E60C4, E2801170000002158BB40D89, E280117000000217F51E61E4, E280117000000217F51E61DF, E2801170000002158BB40D84, E280117000000217F51E719D, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7194</v>
+        <v>E2801170000002158BB40D84, E280117000000217F51E61ED, E280117000000217F51E61DF, E280117000000217F51E61E4, E280117000000217F51E7197, E280117000000217F51E61E7, E2801170000002158BB40D89, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719D</v>
       </c>
       <c r="I35" t="str">
         <v>Source_0, Source_1</v>
@@ -1625,7 +1625,7 @@
         <v>13</v>
       </c>
       <c r="L35" t="str">
-        <v>76.9</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="36">
@@ -1639,28 +1639,28 @@
         <v>35</v>
       </c>
       <c r="D36" t="str">
-        <v>2026-06-02 15:37:57</v>
+        <v>2026-06-02 15:38:50</v>
       </c>
       <c r="E36" t="str">
-        <v>2026-06-02 15:38:12</v>
+        <v>2026-06-02 15:39:05</v>
       </c>
       <c r="F36" t="str">
-        <v>14.34</v>
+        <v>14.55</v>
       </c>
       <c r="G36" t="str">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H36" t="str">
-        <v>E2801170000002158BB40D84, E280117000000217F51E61ED, E280117000000217F51E61DF, E280117000000217F51E61E4, E280117000000217F51E7197, E280117000000217F51E61E7, E2801170000002158BB40D89, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719D</v>
+        <v>E280117000000217F51E60C4, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E7197, E2801170000002158BB40D84, E280117000000217F51E61ED, E280117000000217F51E61E4, E280117000000217F51E61E7, E280117000000217F51E719D, E280117000000217F51E7082, E280117000000217F51E719A, E280117000000217F51E7194, E280117000000217F51E718F</v>
       </c>
       <c r="I36" t="str">
-        <v>Source_0, Source_1</v>
+        <v>Source_1</v>
       </c>
       <c r="K36" t="str">
         <v>13</v>
       </c>
       <c r="L36" t="str">
-        <v>92.3</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37">
@@ -1674,28 +1674,28 @@
         <v>36</v>
       </c>
       <c r="D37" t="str">
-        <v>2026-06-02 15:38:50</v>
+        <v>2026-06-02 15:40:06</v>
       </c>
       <c r="E37" t="str">
-        <v>2026-06-02 15:39:05</v>
+        <v>2026-06-02 15:40:26</v>
       </c>
       <c r="F37" t="str">
-        <v>14.55</v>
+        <v>19.93</v>
       </c>
       <c r="G37" t="str">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H37" t="str">
-        <v>E280117000000217F51E60C4, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E7197, E2801170000002158BB40D84, E280117000000217F51E61ED, E280117000000217F51E61E4, E280117000000217F51E61E7, E280117000000217F51E719D, E280117000000217F51E7082, E280117000000217F51E719A, E280117000000217F51E7194, E280117000000217F51E718F</v>
+        <v>E280117000000217F51E61E7, E280117000000217F51E7197, E280117000000217F51E60C4, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E61ED, E280117000000217F51E61E4, E280117000000217F51E61DF, E2801170000002158BB40D84</v>
       </c>
       <c r="I37" t="str">
-        <v>Source_1</v>
+        <v>Source_0, Source_1</v>
       </c>
       <c r="K37" t="str">
         <v>13</v>
       </c>
       <c r="L37" t="str">
-        <v>100</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="38">
@@ -1709,19 +1709,19 @@
         <v>37</v>
       </c>
       <c r="D38" t="str">
-        <v>2026-06-02 15:40:06</v>
+        <v>2026-06-02 15:40:53</v>
       </c>
       <c r="E38" t="str">
-        <v>2026-06-02 15:40:26</v>
+        <v>2026-06-02 15:41:07</v>
       </c>
       <c r="F38" t="str">
-        <v>19.93</v>
+        <v>13.44</v>
       </c>
       <c r="G38" t="str">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H38" t="str">
-        <v>E280117000000217F51E61E7, E280117000000217F51E7197, E280117000000217F51E60C4, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E61ED, E280117000000217F51E61E4, E280117000000217F51E61DF, E2801170000002158BB40D84</v>
+        <v>E2801170000002158BB40D84, E2801170000002158BB40D89, E280117000000217F51E60C4, E280117000000217F51E61DF, E280117000000217F51E61ED, E280117000000217F51E61E7, E280117000000217F51E61E4, E280117000000217F51E7197, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E7194</v>
       </c>
       <c r="I38" t="str">
         <v>Source_0, Source_1</v>
@@ -1730,7 +1730,7 @@
         <v>13</v>
       </c>
       <c r="L38" t="str">
-        <v>92.3</v>
+        <v>100</v>
       </c>
     </row>
     <row r="39">
@@ -1744,19 +1744,19 @@
         <v>38</v>
       </c>
       <c r="D39" t="str">
-        <v>2026-06-02 15:40:53</v>
+        <v>2026-06-02 15:41:25</v>
       </c>
       <c r="E39" t="str">
-        <v>2026-06-02 15:41:07</v>
+        <v>2026-06-02 15:41:37</v>
       </c>
       <c r="F39" t="str">
-        <v>13.44</v>
+        <v>12.12</v>
       </c>
       <c r="G39" t="str">
         <v>13</v>
       </c>
       <c r="H39" t="str">
-        <v>E2801170000002158BB40D84, E2801170000002158BB40D89, E280117000000217F51E60C4, E280117000000217F51E61DF, E280117000000217F51E61ED, E280117000000217F51E61E7, E280117000000217F51E61E4, E280117000000217F51E7197, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E7194</v>
+        <v>E280117000000217F51E61E4, E280117000000217F51E7197, E280117000000217F51E60C4, E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E61ED, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E719D</v>
       </c>
       <c r="I39" t="str">
         <v>Source_0, Source_1</v>
@@ -1779,19 +1779,19 @@
         <v>39</v>
       </c>
       <c r="D40" t="str">
-        <v>2026-06-02 15:41:25</v>
+        <v>2026-06-02 15:42:46</v>
       </c>
       <c r="E40" t="str">
-        <v>2026-06-02 15:41:37</v>
+        <v>2026-06-02 15:42:59</v>
       </c>
       <c r="F40" t="str">
-        <v>12.12</v>
+        <v>13.01</v>
       </c>
       <c r="G40" t="str">
         <v>13</v>
       </c>
       <c r="H40" t="str">
-        <v>E280117000000217F51E61E4, E280117000000217F51E7197, E280117000000217F51E60C4, E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E61ED, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E719D</v>
+        <v>E280117000000217F51E7082, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E7194, E280117000000217F51E718F, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E61ED, E280117000000217F51E7197, E2801170000002158BB40D84, E280117000000217F51E61E4, E280117000000217F51E61E7, E280117000000217F51E60C4</v>
       </c>
       <c r="I40" t="str">
         <v>Source_0, Source_1</v>
@@ -1814,22 +1814,22 @@
         <v>40</v>
       </c>
       <c r="D41" t="str">
-        <v>2026-06-02 15:42:46</v>
+        <v>2026-06-02 15:43:44</v>
       </c>
       <c r="E41" t="str">
-        <v>2026-06-02 15:42:59</v>
+        <v>2026-06-02 15:43:58</v>
       </c>
       <c r="F41" t="str">
-        <v>13.01</v>
+        <v>13.77</v>
       </c>
       <c r="G41" t="str">
         <v>13</v>
       </c>
       <c r="H41" t="str">
-        <v>E280117000000217F51E7082, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E7194, E280117000000217F51E718F, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E61ED, E280117000000217F51E7197, E2801170000002158BB40D84, E280117000000217F51E61E4, E280117000000217F51E61E7, E280117000000217F51E60C4</v>
+        <v>E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E7197, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E60C4, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E719A, E280117000000217F51E7194, E280117000000217F51E719D</v>
       </c>
       <c r="I41" t="str">
-        <v>Source_0, Source_1</v>
+        <v>Source_1</v>
       </c>
       <c r="K41" t="str">
         <v>13</v>
@@ -1849,22 +1849,22 @@
         <v>41</v>
       </c>
       <c r="D42" t="str">
-        <v>2026-06-02 15:43:44</v>
+        <v>2026-06-02 15:44:39</v>
       </c>
       <c r="E42" t="str">
-        <v>2026-06-02 15:43:58</v>
+        <v>2026-06-02 15:44:53</v>
       </c>
       <c r="F42" t="str">
-        <v>13.77</v>
+        <v>13.55</v>
       </c>
       <c r="G42" t="str">
         <v>13</v>
       </c>
       <c r="H42" t="str">
-        <v>E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E7197, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E60C4, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E719A, E280117000000217F51E7194, E280117000000217F51E719D</v>
+        <v>E280117000000217F51E61DF, E280117000000217F51E60C4, E280117000000217F51E61E4, E2801170000002158BB40D89, E280117000000217F51E7197, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E719D, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E61E7, E2801170000002158BB40D84, E280117000000217F51E61ED</v>
       </c>
       <c r="I42" t="str">
-        <v>Source_1</v>
+        <v>Source_0, Source_1</v>
       </c>
       <c r="K42" t="str">
         <v>13</v>
@@ -1884,19 +1884,19 @@
         <v>42</v>
       </c>
       <c r="D43" t="str">
-        <v>2026-06-02 15:44:39</v>
+        <v>2026-06-02 15:45:43</v>
       </c>
       <c r="E43" t="str">
-        <v>2026-06-02 15:44:53</v>
+        <v>2026-06-02 15:45:58</v>
       </c>
       <c r="F43" t="str">
-        <v>13.55</v>
+        <v>14.67</v>
       </c>
       <c r="G43" t="str">
         <v>13</v>
       </c>
       <c r="H43" t="str">
-        <v>E280117000000217F51E61DF, E280117000000217F51E60C4, E280117000000217F51E61E4, E2801170000002158BB40D89, E280117000000217F51E7197, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E719D, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E61E7, E2801170000002158BB40D84, E280117000000217F51E61ED</v>
+        <v>E280117000000217F51E61ED, E280117000000217F51E60C4, E280117000000217F51E61E7, E2801170000002158BB40D84, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E7197, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E61E4</v>
       </c>
       <c r="I43" t="str">
         <v>Source_0, Source_1</v>
@@ -1910,7 +1910,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>20260602-152458</v>
+        <v>20260602-161257</v>
       </c>
       <c r="B44" t="str">
         <v>antennas_vertical</v>
@@ -1919,22 +1919,22 @@
         <v>43</v>
       </c>
       <c r="D44" t="str">
-        <v>2026-06-02 15:45:43</v>
+        <v>2026-06-02 16:13:16</v>
       </c>
       <c r="E44" t="str">
-        <v>2026-06-02 15:45:58</v>
+        <v>2026-06-02 16:13:36</v>
       </c>
       <c r="F44" t="str">
-        <v>14.67</v>
+        <v>19.7</v>
       </c>
       <c r="G44" t="str">
         <v>13</v>
       </c>
       <c r="H44" t="str">
-        <v>E280117000000217F51E61ED, E280117000000217F51E60C4, E280117000000217F51E61E7, E2801170000002158BB40D84, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E7197, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E61E4</v>
+        <v>E280117000000217F51E61E4, E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E61ED, E280117000000217F51E61E7, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E7194, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E60C4, E280117000000217F51E7197, E2801170000002158BB40D84</v>
       </c>
       <c r="I44" t="str">
-        <v>Source_0, Source_1</v>
+        <v>Source_1</v>
       </c>
       <c r="K44" t="str">
         <v>13</v>
@@ -1954,22 +1954,22 @@
         <v>44</v>
       </c>
       <c r="D45" t="str">
-        <v>2026-06-02 16:13:16</v>
+        <v>2026-06-02 16:15:32</v>
       </c>
       <c r="E45" t="str">
-        <v>2026-06-02 16:13:36</v>
+        <v>2026-06-02 16:15:47</v>
       </c>
       <c r="F45" t="str">
-        <v>19.7</v>
+        <v>14.4</v>
       </c>
       <c r="G45" t="str">
         <v>13</v>
       </c>
       <c r="H45" t="str">
-        <v>E280117000000217F51E61E4, E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E61ED, E280117000000217F51E61E7, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E7194, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E60C4, E280117000000217F51E7197, E2801170000002158BB40D84</v>
+        <v>E280117000000217F51E60C4, E280117000000217F51E61E7, E280117000000217F51E7197, E2801170000002158BB40D84, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E61ED, E280117000000217F51E61E4, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E7194</v>
       </c>
       <c r="I45" t="str">
-        <v>Source_1</v>
+        <v>Source_0, Source_1</v>
       </c>
       <c r="K45" t="str">
         <v>13</v>
@@ -1989,19 +1989,19 @@
         <v>45</v>
       </c>
       <c r="D46" t="str">
-        <v>2026-06-02 16:15:32</v>
+        <v>2026-06-02 16:16:07</v>
       </c>
       <c r="E46" t="str">
-        <v>2026-06-02 16:15:47</v>
+        <v>2026-06-02 16:16:19</v>
       </c>
       <c r="F46" t="str">
-        <v>14.4</v>
+        <v>12.05</v>
       </c>
       <c r="G46" t="str">
         <v>13</v>
       </c>
       <c r="H46" t="str">
-        <v>E280117000000217F51E60C4, E280117000000217F51E61E7, E280117000000217F51E7197, E2801170000002158BB40D84, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E61ED, E280117000000217F51E61E4, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E7194</v>
+        <v>E280117000000217F51E61E4, E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E60C4, E2801170000002158BB40D84, E280117000000217F51E719A, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719D, E280117000000217F51E7197, E280117000000217F51E61ED, E280117000000217F51E61E7</v>
       </c>
       <c r="I46" t="str">
         <v>Source_0, Source_1</v>
@@ -2024,19 +2024,19 @@
         <v>46</v>
       </c>
       <c r="D47" t="str">
-        <v>2026-06-02 16:16:07</v>
+        <v>2026-06-02 16:16:42</v>
       </c>
       <c r="E47" t="str">
-        <v>2026-06-02 16:16:19</v>
+        <v>2026-06-02 16:16:52</v>
       </c>
       <c r="F47" t="str">
-        <v>12.05</v>
+        <v>10.81</v>
       </c>
       <c r="G47" t="str">
         <v>13</v>
       </c>
       <c r="H47" t="str">
-        <v>E280117000000217F51E61E4, E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E60C4, E2801170000002158BB40D84, E280117000000217F51E719A, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719D, E280117000000217F51E7197, E280117000000217F51E61ED, E280117000000217F51E61E7</v>
+        <v>E2801170000002158BB40D89, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E61ED, E280117000000217F51E61E7, E2801170000002158BB40D84, E280117000000217F51E7197, E280117000000217F51E61E4, E280117000000217F51E61DF, E280117000000217F51E60C4</v>
       </c>
       <c r="I47" t="str">
         <v>Source_0, Source_1</v>
@@ -2059,19 +2059,19 @@
         <v>47</v>
       </c>
       <c r="D48" t="str">
-        <v>2026-06-02 16:16:42</v>
+        <v>2026-06-02 16:17:22</v>
       </c>
       <c r="E48" t="str">
-        <v>2026-06-02 16:16:52</v>
+        <v>2026-06-02 16:17:36</v>
       </c>
       <c r="F48" t="str">
-        <v>10.81</v>
+        <v>13.92</v>
       </c>
       <c r="G48" t="str">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H48" t="str">
-        <v>E2801170000002158BB40D89, E280117000000217F51E718F, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E61ED, E280117000000217F51E61E7, E2801170000002158BB40D84, E280117000000217F51E7197, E280117000000217F51E61E4, E280117000000217F51E61DF, E280117000000217F51E60C4</v>
+        <v>E280117000000217F51E61DF, E280117000000217F51E60C4, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E719D, E2801170000002158BB40D89, E280117000000217F51E61ED, E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E61E4</v>
       </c>
       <c r="I48" t="str">
         <v>Source_0, Source_1</v>
@@ -2080,7 +2080,7 @@
         <v>13</v>
       </c>
       <c r="L48" t="str">
-        <v>100</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="49">
@@ -2094,19 +2094,19 @@
         <v>48</v>
       </c>
       <c r="D49" t="str">
-        <v>2026-06-02 16:17:22</v>
+        <v>2026-06-02 16:17:55</v>
       </c>
       <c r="E49" t="str">
-        <v>2026-06-02 16:17:36</v>
+        <v>2026-06-02 16:18:07</v>
       </c>
       <c r="F49" t="str">
-        <v>13.92</v>
+        <v>12.62</v>
       </c>
       <c r="G49" t="str">
         <v>12</v>
       </c>
       <c r="H49" t="str">
-        <v>E280117000000217F51E61DF, E280117000000217F51E60C4, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E719D, E2801170000002158BB40D89, E280117000000217F51E61ED, E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E61E4</v>
+        <v>E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E61ED, E280117000000217F51E61E4, E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E60C4, E280117000000217F51E7082, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E718F, E280117000000217F51E7194</v>
       </c>
       <c r="I49" t="str">
         <v>Source_0, Source_1</v>
@@ -2120,7 +2120,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>20260602-161257</v>
+        <v>20260602-163046</v>
       </c>
       <c r="B50" t="str">
         <v>antennas_vertical</v>
@@ -2129,19 +2129,19 @@
         <v>49</v>
       </c>
       <c r="D50" t="str">
-        <v>2026-06-02 16:17:55</v>
+        <v>2026-06-02 16:31:00</v>
       </c>
       <c r="E50" t="str">
-        <v>2026-06-02 16:18:07</v>
+        <v>2026-06-02 16:31:14</v>
       </c>
       <c r="F50" t="str">
-        <v>12.62</v>
+        <v>14.04</v>
       </c>
       <c r="G50" t="str">
         <v>12</v>
       </c>
       <c r="H50" t="str">
-        <v>E2801170000002158BB40D84, E280117000000217F51E61E7, E280117000000217F51E61ED, E280117000000217F51E61E4, E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E60C4, E280117000000217F51E7082, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E718F, E280117000000217F51E7194</v>
+        <v>E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E7194, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E61E7, E280117000000217F51E60C4, E2801170000002158BB40D84</v>
       </c>
       <c r="I50" t="str">
         <v>Source_0, Source_1</v>
@@ -2153,44 +2153,9 @@
         <v>92.3</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="str">
-        <v>20260602-163046</v>
-      </c>
-      <c r="B51" t="str">
-        <v>antennas_vertical</v>
-      </c>
-      <c r="C51" t="str">
-        <v>50</v>
-      </c>
-      <c r="D51" t="str">
-        <v>2026-06-02 16:31:00</v>
-      </c>
-      <c r="E51" t="str">
-        <v>2026-06-02 16:31:14</v>
-      </c>
-      <c r="F51" t="str">
-        <v>14.04</v>
-      </c>
-      <c r="G51" t="str">
-        <v>12</v>
-      </c>
-      <c r="H51" t="str">
-        <v>E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E7082, E280117000000217F51E718F, E280117000000217F51E7194, E2801170000002158BB40D89, E280117000000217F51E61DF, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E61E7, E280117000000217F51E60C4, E2801170000002158BB40D84</v>
-      </c>
-      <c r="I51" t="str">
-        <v>Source_0, Source_1</v>
-      </c>
-      <c r="K51" t="str">
-        <v>13</v>
-      </c>
-      <c r="L51" t="str">
-        <v>92.3</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L50"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Test results from Pi 2026-06-03_11-09
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -1543,6 +1543,202 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>101</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1019175" cy="762000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="52" name="Image 52" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId52"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>102</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1019175" cy="762000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="53" name="Image 53" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId53"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>103</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1019175" cy="762000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="54" name="Image 54" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId54"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>104</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1019175" cy="762000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="55" name="Image 55" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId55"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>105</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1019175" cy="762000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="56" name="Image 56" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId56"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>106</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1019175" cy="762000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="57" name="Image 57" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId57"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>107</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1019175" cy="762000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="58" name="Image 58" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId58"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1876,7 +2072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L101"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7108,12 +7304,341 @@
           <t>Source_0, Source_1</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr"/>
       <c r="K101" t="n">
         <v>13</v>
       </c>
       <c r="L101" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="102" ht="64" customHeight="1">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>1</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:55:54</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:56:53</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>59.27</v>
+      </c>
+      <c r="G102" t="n">
+        <v>6</v>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E60C4, E280117000000217F51E61E4, E280117000000217F51E61E7, E280117000000217F51E61ED, E2801170000002158BB40D84, E280117000000217F51E7197</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="K102" t="n">
+        <v>13</v>
+      </c>
+      <c r="L102" t="n">
+        <v>46.2</v>
+      </c>
+    </row>
+    <row r="103" ht="64" customHeight="1">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>2</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:57:10</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:57:26</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>15.72</v>
+      </c>
+      <c r="G103" t="n">
+        <v>13</v>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7197, E280117000000217F51E61DF, E2801170000002158BB40D89, E280117000000217F51E61E4, E280117000000217F51E61ED, E280117000000217F51E719A, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E718F, E280117000000217F51E719D, E280117000000217F51E60C4, E280117000000217F51E61E7, E2801170000002158BB40D84</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Source_0, Source_1</t>
+        </is>
+      </c>
+      <c r="K103" t="n">
+        <v>13</v>
+      </c>
+      <c r="L103" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="104" ht="64" customHeight="1">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>3</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:58:23</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:58:38</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>15.09</v>
+      </c>
+      <c r="G104" t="n">
+        <v>13</v>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61E7, E2801170000002158BB40D89, E280117000000217F51E61ED, E280117000000217F51E719D, E280117000000217F51E719A, E280117000000217F51E718F, E280117000000217F51E7194, E280117000000217F51E7082, E280117000000217F51E61DF, E280117000000217F51E60C4, E280117000000217F51E7197, E280117000000217F51E61E4, E2801170000002158BB40D84</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Source_0, Source_1</t>
+        </is>
+      </c>
+      <c r="K104" t="n">
+        <v>13</v>
+      </c>
+      <c r="L104" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="105" ht="64" customHeight="1">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>4</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:59:36</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:59:57</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>21.22</v>
+      </c>
+      <c r="G105" t="n">
+        <v>9</v>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>E2801170000002158BB40D84, E280117000000217F51E7197, E280117000000217F51E60C4, E280117000000217F51E61E7, E280117000000217F51E718F, E280117000000217F51E7194, E280117000000217F51E7082, E280117000000217F51E719A, E280117000000217F51E719D</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Source_0, Source_1</t>
+        </is>
+      </c>
+      <c r="K105" t="n">
+        <v>13</v>
+      </c>
+      <c r="L105" t="n">
+        <v>69.2</v>
+      </c>
+    </row>
+    <row r="106" ht="64" customHeight="1">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>5</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:00:34</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:00:45</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>11.69</v>
+      </c>
+      <c r="G106" t="n">
+        <v>13</v>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E718F, E280117000000217F51E61E7, E280117000000217F51E61ED, E2801170000002158BB40D89, E280117000000217F51E61E4, E280117000000217F51E7197, E280117000000217F51E61DF, E280117000000217F51E60C4, E2801170000002158BB40D84</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Source_0, Source_1</t>
+        </is>
+      </c>
+      <c r="K106" t="n">
+        <v>13</v>
+      </c>
+      <c r="L106" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="107" ht="64" customHeight="1">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>6</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:01:25</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:01:37</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>11.23</v>
+      </c>
+      <c r="G107" t="n">
+        <v>13</v>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61DF, E280117000000217F51E61ED, E280117000000217F51E60C4, E280117000000217F51E7197, E280117000000217F51E61E4, E2801170000002158BB40D89, E280117000000217F51E61E7, E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E719D, E280117000000217F51E718F, E280117000000217F51E719A, E2801170000002158BB40D84</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Source_0, Source_1</t>
+        </is>
+      </c>
+      <c r="K107" t="n">
+        <v>13</v>
+      </c>
+      <c r="L107" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="108" ht="64" customHeight="1">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>7</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:03:40</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:03:53</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="G108" t="n">
+        <v>7</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7082, E280117000000217F51E7194, E280117000000217F51E718F, E280117000000217F51E719A, E280117000000217F51E719D, E280117000000217F51E61E4, E2801170000002158BB40D84</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Source_0, Source_1</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="n">
+        <v>13</v>
+      </c>
+      <c r="L108" t="n">
+        <v>53.8</v>
       </c>
     </row>
   </sheetData>
@@ -7128,7 +7653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1265"/>
+  <dimension ref="A1:F1339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46351,6 +46876,2226 @@
         </is>
       </c>
     </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1266" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1266" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E60C4</t>
+        </is>
+      </c>
+      <c r="E1266" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1266" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:55:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1267" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1267" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61E4</t>
+        </is>
+      </c>
+      <c r="E1267" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1267" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:55:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1268" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1268" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61E7</t>
+        </is>
+      </c>
+      <c r="E1268" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1268" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:56:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1269" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1269" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61ED</t>
+        </is>
+      </c>
+      <c r="E1269" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1269" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:56:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1270" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1270" t="inlineStr">
+        <is>
+          <t>E2801170000002158BB40D84</t>
+        </is>
+      </c>
+      <c r="E1270" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1270" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:56:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1271" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1271" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7197</t>
+        </is>
+      </c>
+      <c r="E1271" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1271" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:56:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1272" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1272" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7197</t>
+        </is>
+      </c>
+      <c r="E1272" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1272" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:57:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1273" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1273" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61DF</t>
+        </is>
+      </c>
+      <c r="E1273" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1273" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:57:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1274" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1274" t="inlineStr">
+        <is>
+          <t>E2801170000002158BB40D89</t>
+        </is>
+      </c>
+      <c r="E1274" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1274" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:57:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1275" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1275" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61E4</t>
+        </is>
+      </c>
+      <c r="E1275" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1275" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:57:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1276" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1276" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61ED</t>
+        </is>
+      </c>
+      <c r="E1276" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1276" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:57:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1277" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1277" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E719A</t>
+        </is>
+      </c>
+      <c r="E1277" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1277" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:57:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1278" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1278" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7082</t>
+        </is>
+      </c>
+      <c r="E1278" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1278" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:57:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1279" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1279" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7194</t>
+        </is>
+      </c>
+      <c r="E1279" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1279" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:57:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1280" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1280" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E718F</t>
+        </is>
+      </c>
+      <c r="E1280" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1280" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:57:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1281" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1281" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E719D</t>
+        </is>
+      </c>
+      <c r="E1281" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1281" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:57:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1282" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1282" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E60C4</t>
+        </is>
+      </c>
+      <c r="E1282" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1282" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:57:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1283" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1283" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61E7</t>
+        </is>
+      </c>
+      <c r="E1283" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1283" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:57:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1284" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1284" t="inlineStr">
+        <is>
+          <t>E2801170000002158BB40D84</t>
+        </is>
+      </c>
+      <c r="E1284" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1284" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:57:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1285" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1285" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61E7</t>
+        </is>
+      </c>
+      <c r="E1285" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1285" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:58:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1286" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1286" t="inlineStr">
+        <is>
+          <t>E2801170000002158BB40D89</t>
+        </is>
+      </c>
+      <c r="E1286" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1286" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:58:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1287" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1287" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61ED</t>
+        </is>
+      </c>
+      <c r="E1287" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1287" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:58:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1288" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1288" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E719D</t>
+        </is>
+      </c>
+      <c r="E1288" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1288" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:58:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1289" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1289" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E719A</t>
+        </is>
+      </c>
+      <c r="E1289" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1289" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:58:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1290" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1290" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E718F</t>
+        </is>
+      </c>
+      <c r="E1290" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1290" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:58:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1291" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1291" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7194</t>
+        </is>
+      </c>
+      <c r="E1291" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1291" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:58:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1292" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1292" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7082</t>
+        </is>
+      </c>
+      <c r="E1292" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1292" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:58:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1293" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1293" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61DF</t>
+        </is>
+      </c>
+      <c r="E1293" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1293" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:58:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1294" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1294" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E60C4</t>
+        </is>
+      </c>
+      <c r="E1294" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1294" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:58:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1295" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1295" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7197</t>
+        </is>
+      </c>
+      <c r="E1295" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1295" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:58:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1296" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1296" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61E4</t>
+        </is>
+      </c>
+      <c r="E1296" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1296" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:58:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1297" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1297" t="inlineStr">
+        <is>
+          <t>E2801170000002158BB40D84</t>
+        </is>
+      </c>
+      <c r="E1297" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1297" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:58:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1298" t="n">
+        <v>4</v>
+      </c>
+      <c r="D1298" t="inlineStr">
+        <is>
+          <t>E2801170000002158BB40D84</t>
+        </is>
+      </c>
+      <c r="E1298" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1298" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:59:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1299" t="n">
+        <v>4</v>
+      </c>
+      <c r="D1299" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7197</t>
+        </is>
+      </c>
+      <c r="E1299" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1299" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:59:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1300" t="n">
+        <v>4</v>
+      </c>
+      <c r="D1300" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E60C4</t>
+        </is>
+      </c>
+      <c r="E1300" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1300" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:59:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1301" t="n">
+        <v>4</v>
+      </c>
+      <c r="D1301" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61E7</t>
+        </is>
+      </c>
+      <c r="E1301" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1301" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:59:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1302" t="n">
+        <v>4</v>
+      </c>
+      <c r="D1302" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E718F</t>
+        </is>
+      </c>
+      <c r="E1302" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1302" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:59:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1303" t="n">
+        <v>4</v>
+      </c>
+      <c r="D1303" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7194</t>
+        </is>
+      </c>
+      <c r="E1303" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1303" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:59:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1304" t="n">
+        <v>4</v>
+      </c>
+      <c r="D1304" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7082</t>
+        </is>
+      </c>
+      <c r="E1304" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1304" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:59:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1305" t="n">
+        <v>4</v>
+      </c>
+      <c r="D1305" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E719A</t>
+        </is>
+      </c>
+      <c r="E1305" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1305" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:59:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1306" t="n">
+        <v>4</v>
+      </c>
+      <c r="D1306" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E719D</t>
+        </is>
+      </c>
+      <c r="E1306" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1306" t="inlineStr">
+        <is>
+          <t>2026-06-03 10:59:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1307" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1307" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7082</t>
+        </is>
+      </c>
+      <c r="E1307" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1307" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:00:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1308" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1308" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7194</t>
+        </is>
+      </c>
+      <c r="E1308" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1308" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:00:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1309" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1309" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E719A</t>
+        </is>
+      </c>
+      <c r="E1309" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1309" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:00:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1310" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1310" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E719D</t>
+        </is>
+      </c>
+      <c r="E1310" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1310" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:00:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1311" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1311" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E718F</t>
+        </is>
+      </c>
+      <c r="E1311" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1311" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:00:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1312" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1312" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61E7</t>
+        </is>
+      </c>
+      <c r="E1312" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1312" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:00:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1313" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1313" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61ED</t>
+        </is>
+      </c>
+      <c r="E1313" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1313" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:00:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1314" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1314" t="inlineStr">
+        <is>
+          <t>E2801170000002158BB40D89</t>
+        </is>
+      </c>
+      <c r="E1314" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1314" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:00:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1315" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1315" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61E4</t>
+        </is>
+      </c>
+      <c r="E1315" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1315" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:00:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1316" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1316" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7197</t>
+        </is>
+      </c>
+      <c r="E1316" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1316" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:00:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1317" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1317" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61DF</t>
+        </is>
+      </c>
+      <c r="E1317" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1317" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:00:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1318" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1318" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E60C4</t>
+        </is>
+      </c>
+      <c r="E1318" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1318" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:00:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1319" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1319" t="inlineStr">
+        <is>
+          <t>E2801170000002158BB40D84</t>
+        </is>
+      </c>
+      <c r="E1319" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1319" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:00:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1320" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1320" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61DF</t>
+        </is>
+      </c>
+      <c r="E1320" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1320" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:01:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1321" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1321" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61ED</t>
+        </is>
+      </c>
+      <c r="E1321" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1321" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:01:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1322" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1322" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E60C4</t>
+        </is>
+      </c>
+      <c r="E1322" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1322" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:01:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1323" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1323" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7197</t>
+        </is>
+      </c>
+      <c r="E1323" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1323" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:01:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1324" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1324" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61E4</t>
+        </is>
+      </c>
+      <c r="E1324" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1324" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:01:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1325" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1325" t="inlineStr">
+        <is>
+          <t>E2801170000002158BB40D89</t>
+        </is>
+      </c>
+      <c r="E1325" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1325" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:01:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1326" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1326" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61E7</t>
+        </is>
+      </c>
+      <c r="E1326" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1326" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:01:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1327" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1327" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7082</t>
+        </is>
+      </c>
+      <c r="E1327" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1327" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:01:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1328" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1328" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7194</t>
+        </is>
+      </c>
+      <c r="E1328" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1328" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:01:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1329" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1329" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E719D</t>
+        </is>
+      </c>
+      <c r="E1329" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1329" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:01:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1330" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1330" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E718F</t>
+        </is>
+      </c>
+      <c r="E1330" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1330" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:01:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1331" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1331" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E719A</t>
+        </is>
+      </c>
+      <c r="E1331" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1331" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:01:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1332" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1332" t="inlineStr">
+        <is>
+          <t>E2801170000002158BB40D84</t>
+        </is>
+      </c>
+      <c r="E1332" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1332" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:01:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1333" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1333" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7082</t>
+        </is>
+      </c>
+      <c r="E1333" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1333" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:03:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1334" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1334" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E7194</t>
+        </is>
+      </c>
+      <c r="E1334" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1334" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:03:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1335" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1335" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E718F</t>
+        </is>
+      </c>
+      <c r="E1335" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1335" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:03:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1336" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1336" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E719A</t>
+        </is>
+      </c>
+      <c r="E1336" t="inlineStr">
+        <is>
+          <t>Source_0</t>
+        </is>
+      </c>
+      <c r="F1336" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:03:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1337" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E719D</t>
+        </is>
+      </c>
+      <c r="E1337" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1337" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:03:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1338" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>E280117000000217F51E61E4</t>
+        </is>
+      </c>
+      <c r="E1338" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1338" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:03:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr">
+        <is>
+          <t>20260603-105246</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>antennas_opposite</t>
+        </is>
+      </c>
+      <c r="C1339" t="n">
+        <v>7</v>
+      </c>
+      <c r="D1339" t="inlineStr">
+        <is>
+          <t>E2801170000002158BB40D84</t>
+        </is>
+      </c>
+      <c r="E1339" t="inlineStr">
+        <is>
+          <t>Source_1</t>
+        </is>
+      </c>
+      <c r="F1339" t="inlineStr">
+        <is>
+          <t>2026-06-03 11:03:42</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>